<commit_message>
fix: make copyright of photo portrait non mandatory
</commit_message>
<xml_diff>
--- a/src/app/modules/kyc/kyc_models/MVP-2-KYC-Commons-45.xlsx
+++ b/src/app/modules/kyc/kyc_models/MVP-2-KYC-Commons-45.xlsx
@@ -3011,39 +3011,39 @@
         <v>106</v>
       </c>
       <c r="K11" s="41"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="5"/>
-      <c r="W11" s="5"/>
-      <c r="X11" s="5"/>
-      <c r="Y11" s="5"/>
-      <c r="Z11" s="5"/>
-      <c r="AA11" s="5"/>
-      <c r="AB11" s="5"/>
-      <c r="AC11" s="5"/>
-      <c r="AD11" s="5"/>
-      <c r="AE11" s="5"/>
-      <c r="AF11" s="5"/>
-      <c r="AG11" s="5"/>
-      <c r="AH11" s="5"/>
-      <c r="AI11" s="5"/>
-      <c r="AJ11" s="5"/>
-      <c r="AK11" s="5"/>
-      <c r="AL11" s="5"/>
-      <c r="AM11" s="5"/>
-      <c r="AN11" s="5"/>
-      <c r="AO11" s="5"/>
-      <c r="AP11" s="5"/>
-      <c r="AQ11" s="5"/>
-      <c r="AR11" s="5"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7"/>
+      <c r="AA11" s="7"/>
+      <c r="AB11" s="7"/>
+      <c r="AC11" s="7"/>
+      <c r="AD11" s="7"/>
+      <c r="AE11" s="7"/>
+      <c r="AF11" s="7"/>
+      <c r="AG11" s="7"/>
+      <c r="AH11" s="7"/>
+      <c r="AI11" s="7"/>
+      <c r="AJ11" s="7"/>
+      <c r="AK11" s="7"/>
+      <c r="AL11" s="7"/>
+      <c r="AM11" s="7"/>
+      <c r="AN11" s="7"/>
+      <c r="AO11" s="7"/>
+      <c r="AP11" s="7"/>
+      <c r="AQ11" s="7"/>
+      <c r="AR11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">

</xml_diff>